<commit_message>
Update 9-zone PJM data to EPA 2025 Ref Case and finalize 21-zone dataset
- Sync 9-zone PJM data with the most recent EPA 2025 Reference Case.
- Add complete PJM 21-zone dataset, including transmission topology derived from NREL ReEDS.
- Map existing generating units and interconnection queue projects to the 21 zones.
- Restructure 21-zone files directly into `PJM 21 Zone.zip` (generators, lines, interface, queue, load, availability factors).
- Update README with the new 21-zone file list and mapping methodology.
</commit_message>
<xml_diff>
--- a/data/output/IPM Regions_State_Utilities.xlsx
+++ b/data/output/IPM Regions_State_Utilities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skhanal/Desktop/ICARUS-PJM-Dataset/data/raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/skhanal/Desktop/ICARUS-PJM-Dataset/data/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00021B3E-D272-B244-B93F-39EB8C74F3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E666D2-F3B5-1346-AFD4-147B2E5266F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{A087CEB7-F347-0646-AF03-1E1E4342A10E}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{A087CEB7-F347-0646-AF03-1E1E4342A10E}"/>
   </bookViews>
   <sheets>
     <sheet name="IPM Regions to LDAs and Zones" sheetId="3" r:id="rId1"/>
@@ -1474,7 +1474,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="30" x14ac:knownFonts="1">
+  <fonts count="30">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2384,7 +2384,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A8ED6D6-6ACA-514C-860A-16FEA9439F48}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:S65"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="53.1640625" customWidth="1"/>
@@ -2396,7 +2396,7 @@
     <col min="10" max="10" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" s="33" t="s">
         <v>9</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="17">
       <c r="A2" s="38" t="s">
         <v>2</v>
       </c>
@@ -2464,7 +2464,7 @@
         <v>AE</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="17">
       <c r="A3" s="38" t="s">
         <v>8</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>PS</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12">
       <c r="A4" s="38" t="s">
         <v>8</v>
       </c>
@@ -2532,7 +2532,7 @@
         <v>PECO</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12">
       <c r="A5" s="38" t="s">
         <v>8</v>
       </c>
@@ -2566,7 +2566,7 @@
         <v>JCPL</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12">
       <c r="A6" s="38" t="s">
         <v>0</v>
       </c>
@@ -2600,7 +2600,7 @@
         <v>DPL</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12">
       <c r="A7" s="38" t="s">
         <v>1</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>RECO</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12">
       <c r="A8" s="38" t="s">
         <v>8</v>
       </c>
@@ -2659,7 +2659,7 @@
       <c r="I8" s="29"/>
       <c r="K8" s="30"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12">
       <c r="A9" s="38" t="s">
         <v>8</v>
       </c>
@@ -2695,7 +2695,7 @@
         <v>BGE</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12">
       <c r="A10" s="38" t="s">
         <v>8</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>PEPCO</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12">
       <c r="A11" s="38" t="s">
         <v>3</v>
       </c>
@@ -2753,7 +2753,7 @@
       <c r="I11" s="29"/>
       <c r="K11" s="30"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12">
       <c r="A12" s="38" t="s">
         <v>7</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>METED</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12">
       <c r="A13" s="38" t="s">
         <v>7</v>
       </c>
@@ -2824,7 +2824,7 @@
         <v>PL</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12">
       <c r="A14" s="38" t="s">
         <v>5</v>
       </c>
@@ -2849,7 +2849,7 @@
       <c r="I14" s="29"/>
       <c r="K14" s="30"/>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" ht="17">
       <c r="A15" s="38" t="s">
         <v>4</v>
       </c>
@@ -2885,7 +2885,7 @@
         <v>AEP</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" ht="17">
       <c r="A16" s="38" t="s">
         <v>4</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>DAY</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:18" ht="17">
       <c r="A17" s="38" t="s">
         <v>4</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>DLCO</v>
       </c>
     </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:18" ht="17">
       <c r="A18" s="38" t="s">
         <v>4</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>DEOK</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:18" ht="17">
       <c r="A19" s="38" t="s">
         <v>4</v>
       </c>
@@ -3021,7 +3021,7 @@
         <v>EKPC</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:18" ht="17">
       <c r="A20" s="38" t="s">
         <v>4</v>
       </c>
@@ -3053,7 +3053,7 @@
         <v>OVEC</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:18">
       <c r="A21" s="38" t="s">
         <v>6</v>
       </c>
@@ -3079,7 +3079,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:18">
       <c r="A22" s="38" t="s">
         <v>6</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:18" hidden="1">
       <c r="A23" s="29"/>
       <c r="B23" s="22" t="s">
         <v>112</v>
@@ -3123,7 +3123,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:18" hidden="1">
       <c r="A24" s="38" t="s">
         <v>1</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:18" hidden="1">
       <c r="A25" s="29"/>
       <c r="B25" s="24" t="s">
         <v>95</v>
@@ -3167,7 +3167,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:18" hidden="1">
       <c r="A26" s="29"/>
       <c r="B26" s="41" t="s">
         <v>97</v>
@@ -3188,7 +3188,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="17" hidden="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:18" hidden="1">
       <c r="A27" s="29"/>
       <c r="B27" s="24" t="s">
         <v>94</v>
@@ -3209,7 +3209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:18" ht="17" hidden="1">
       <c r="A28" s="38" t="s">
         <v>4</v>
       </c>
@@ -3232,7 +3232,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:18" ht="17" hidden="1">
       <c r="A29" s="38" t="s">
         <v>4</v>
       </c>
@@ -3255,7 +3255,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:18" hidden="1">
       <c r="A30" s="31"/>
       <c r="B30" s="47" t="s">
         <v>96</v>
@@ -3276,17 +3276,17 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:18" hidden="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:18" hidden="1">
       <c r="A31" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:18">
       <c r="R32" s="21" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="33" spans="18:19">
       <c r="R33" t="s">
         <v>118</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="34" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="34" spans="18:19">
       <c r="R34" t="s">
         <v>69</v>
       </c>
@@ -3302,7 +3302,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="35" spans="18:19">
       <c r="R35" t="s">
         <v>10</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="36" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="36" spans="18:19">
       <c r="R36" t="s">
         <v>11</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="37" spans="18:19">
       <c r="R37" t="s">
         <v>29</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="38" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="38" spans="18:19">
       <c r="R38" t="s">
         <v>12</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="39" spans="18:19">
       <c r="R39" t="s">
         <v>13</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="40" spans="18:19">
       <c r="R40" t="s">
         <v>14</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="41" spans="18:19">
       <c r="R41" t="s">
         <v>15</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="42" spans="18:19">
       <c r="R42" t="s">
         <v>16</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="43" spans="18:19">
       <c r="R43" t="s">
         <v>17</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="44" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="44" spans="18:19">
       <c r="R44" t="s">
         <v>18</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="45" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="45" spans="18:19">
       <c r="R45" t="s">
         <v>19</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="46" spans="18:19">
       <c r="R46" t="s">
         <v>20</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="47" spans="18:19">
       <c r="R47" t="s">
         <v>21</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="48" spans="18:19" x14ac:dyDescent="0.2">
+    <row r="48" spans="18:19">
       <c r="R48" t="s">
         <v>22</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:19">
       <c r="R49" t="s">
         <v>28</v>
       </c>
@@ -3422,7 +3422,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:19">
       <c r="R50" t="s">
         <v>23</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:19">
       <c r="R51" t="s">
         <v>24</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:19">
       <c r="R52" t="s">
         <v>25</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:19">
       <c r="R53" t="s">
         <v>26</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:19">
       <c r="A54" s="21" t="s">
         <v>123</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:19">
       <c r="A56" s="2" t="s">
         <v>51</v>
       </c>
@@ -3476,7 +3476,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:19">
       <c r="A57" s="2" t="s">
         <v>54</v>
       </c>
@@ -3487,7 +3487,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:19">
       <c r="A58" s="2" t="s">
         <v>57</v>
       </c>
@@ -3498,7 +3498,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:19">
       <c r="A59" s="2" t="s">
         <v>60</v>
       </c>
@@ -3509,7 +3509,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:19">
       <c r="A60" s="2" t="s">
         <v>63</v>
       </c>
@@ -3520,7 +3520,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:19">
       <c r="A61" s="2" t="s">
         <v>66</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:19">
       <c r="A62" s="2" t="s">
         <v>69</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:19">
       <c r="A63" s="2" t="s">
         <v>11</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:19">
       <c r="A64" s="2" t="s">
         <v>74</v>
       </c>
@@ -3564,7 +3564,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3">
       <c r="A65" s="2" t="s">
         <v>77</v>
       </c>
@@ -3590,9 +3590,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3E85E5D-85E3-974C-9D41-378B6EBDF1BA}">
   <dimension ref="A1:Z29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:26">
       <c r="B1" s="5" t="s">
         <v>80</v>
       </c>
@@ -3605,7 +3605,7 @@
       <c r="K1" s="6"/>
       <c r="L1" s="6"/>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:26">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3643,7 +3643,7 @@
         <v>2031</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:26">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>9120</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:26">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -3719,7 +3719,7 @@
         <v>12731</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:26">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>21146</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:26">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -3798,7 +3798,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:26">
       <c r="A7" s="64" t="s">
         <v>4</v>
       </c>
@@ -3886,7 +3886,7 @@
         <v>8.5790538422236648E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:26">
       <c r="A8" s="64"/>
       <c r="B8" s="7" t="s">
         <v>15</v>
@@ -3970,7 +3970,7 @@
         <v>0.12702879529453312</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:26">
       <c r="A9" s="64"/>
       <c r="B9" s="7" t="s">
         <v>20</v>
@@ -4054,7 +4054,7 @@
         <v>0.19285810518419838</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:26">
       <c r="A10" s="64"/>
       <c r="B10" s="7" t="s">
         <v>23</v>
@@ -4138,7 +4138,7 @@
         <v>0.2630234003623545</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:26">
       <c r="A11" s="64"/>
       <c r="B11" s="7" t="s">
         <v>84</v>
@@ -4222,7 +4222,7 @@
         <v>0.31876587665286044</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:26">
       <c r="A12" s="64"/>
       <c r="B12" s="7" t="s">
         <v>27</v>
@@ -4306,7 +4306,7 @@
         <v>1.2533284083816936E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:26">
       <c r="A13" t="s">
         <v>5</v>
       </c>
@@ -4345,7 +4345,7 @@
       </c>
       <c r="Z13" s="19"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:26">
       <c r="A14" s="64" t="s">
         <v>6</v>
       </c>
@@ -4433,7 +4433,7 @@
         <v>0.52321670099357653</v>
       </c>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:26">
       <c r="A15" s="64"/>
       <c r="B15" s="7" t="s">
         <v>25</v>
@@ -4517,7 +4517,7 @@
         <v>0.47678329900642347</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:26">
       <c r="A16" s="64" t="s">
         <v>7</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>0.29032707246743084</v>
       </c>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:26">
       <c r="A17" s="64"/>
       <c r="B17" s="12" t="s">
         <v>83</v>
@@ -4689,7 +4689,7 @@
         <v>0.70967292753256916</v>
       </c>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:26">
       <c r="A18" s="64" t="s">
         <v>8</v>
       </c>
@@ -4777,7 +4777,7 @@
         <v>0.6209763257023484</v>
       </c>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:26">
       <c r="A19" s="64"/>
       <c r="B19" s="7" t="s">
         <v>14</v>
@@ -4861,7 +4861,7 @@
         <v>9.1035390040308167E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:26">
       <c r="A20" s="64"/>
       <c r="B20" s="8" t="s">
         <v>17</v>
@@ -4945,7 +4945,7 @@
         <v>0.14798640419137671</v>
       </c>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:26">
       <c r="A21" s="64"/>
       <c r="B21" s="7" t="s">
         <v>18</v>
@@ -5029,7 +5029,7 @@
         <v>7.7469870762216231E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:26">
       <c r="A22" s="64"/>
       <c r="B22" s="7" t="s">
         <v>19</v>
@@ -5113,7 +5113,7 @@
         <v>6.0062068398231014E-2</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:26">
       <c r="A23" s="64"/>
       <c r="B23" s="7" t="s">
         <v>22</v>
@@ -5197,7 +5197,7 @@
         <v>2.4699409055194627E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:26">
       <c r="B24" s="12" t="s">
         <v>85</v>
       </c>
@@ -5232,7 +5232,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:26">
       <c r="B25" s="9" t="s">
         <v>87</v>
       </c>
@@ -5267,7 +5267,7 @@
         <v>160512.9049283551</v>
       </c>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:26">
       <c r="B26" s="9" t="s">
         <v>88</v>
       </c>
@@ -5302,7 +5302,7 @@
         <v>10492</v>
       </c>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:26">
       <c r="B29" t="s">
         <v>89</v>
       </c>
@@ -5356,7 +5356,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41B30492-09A7-B54B-8967-B2868E8D631F}">
   <dimension ref="A1:J41"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="46.1640625" bestFit="1" customWidth="1"/>
@@ -5365,12 +5365,12 @@
     <col min="10" max="10" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="54" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10">
       <c r="A2" s="52" t="s">
         <v>129</v>
       </c>
@@ -5399,7 +5399,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="17">
       <c r="A3" s="29" t="s">
         <v>29</v>
       </c>
@@ -5429,7 +5429,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10">
       <c r="A4" s="29" t="s">
         <v>10</v>
       </c>
@@ -5459,7 +5459,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10">
       <c r="A5" s="29" t="s">
         <v>10</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10">
       <c r="A6" s="29" t="s">
         <v>10</v>
       </c>
@@ -5519,7 +5519,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10">
       <c r="A7" s="29" t="s">
         <v>10</v>
       </c>
@@ -5549,7 +5549,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10">
       <c r="A8" s="29" t="s">
         <v>10</v>
       </c>
@@ -5579,7 +5579,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10">
       <c r="A9" s="29" t="s">
         <v>10</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10">
       <c r="A10" s="29" t="s">
         <v>10</v>
       </c>
@@ -5639,7 +5639,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10">
       <c r="A11" s="29" t="s">
         <v>69</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10">
       <c r="A12" s="29" t="s">
         <v>69</v>
       </c>
@@ -5699,7 +5699,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10">
       <c r="A13" s="29" t="s">
         <v>69</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10">
       <c r="A14" s="29" t="s">
         <v>69</v>
       </c>
@@ -5759,7 +5759,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10">
       <c r="A15" s="29" t="s">
         <v>11</v>
       </c>
@@ -5789,7 +5789,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="17">
       <c r="A16" s="29" t="s">
         <v>11</v>
       </c>
@@ -5819,7 +5819,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="17">
       <c r="A17" s="29" t="s">
         <v>12</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="17">
       <c r="A18" s="29" t="s">
         <v>86</v>
       </c>
@@ -5879,7 +5879,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="17">
       <c r="A19" s="29" t="s">
         <v>14</v>
       </c>
@@ -5909,7 +5909,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="17">
       <c r="A20" s="29" t="s">
         <v>17</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="17">
       <c r="A21" s="29" t="s">
         <v>17</v>
       </c>
@@ -5969,7 +5969,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10">
       <c r="A22" s="29" t="s">
         <v>18</v>
       </c>
@@ -5999,7 +5999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10">
       <c r="A23" s="29" t="s">
         <v>77</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10">
       <c r="A24" s="29" t="s">
         <v>77</v>
       </c>
@@ -6050,7 +6050,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="17">
       <c r="A25" s="29" t="s">
         <v>15</v>
       </c>
@@ -6071,7 +6071,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="17">
       <c r="A26" s="29" t="s">
         <v>15</v>
       </c>
@@ -6092,7 +6092,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="17">
       <c r="A27" s="29" t="s">
         <v>15</v>
       </c>
@@ -6113,7 +6113,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10">
       <c r="A28" s="29" t="s">
         <v>19</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="17">
       <c r="A29" s="29" t="s">
         <v>20</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10">
       <c r="A30" s="29" t="s">
         <v>21</v>
       </c>
@@ -6176,7 +6176,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10">
       <c r="A31" s="29" t="s">
         <v>22</v>
       </c>
@@ -6197,7 +6197,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="17">
       <c r="A32" s="29" t="s">
         <v>23</v>
       </c>
@@ -6218,7 +6218,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7">
       <c r="A33" s="29" t="s">
         <v>82</v>
       </c>
@@ -6239,7 +6239,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7">
       <c r="A34" s="29" t="s">
         <v>25</v>
       </c>
@@ -6261,7 +6261,7 @@
       </c>
       <c r="G34" s="11"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7">
       <c r="A35" s="29" t="s">
         <v>25</v>
       </c>
@@ -6282,7 +6282,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7">
       <c r="A36" s="29" t="s">
         <v>83</v>
       </c>
@@ -6303,7 +6303,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" ht="17">
       <c r="A37" s="29" t="s">
         <v>84</v>
       </c>
@@ -6324,7 +6324,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" ht="17">
       <c r="A38" s="29" t="s">
         <v>27</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7">
       <c r="A39" s="29" t="s">
         <v>85</v>
       </c>
@@ -6366,7 +6366,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7">
       <c r="A40" s="59" t="s">
         <v>88</v>
       </c>
@@ -6381,7 +6381,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7">
       <c r="A41" s="60" t="s">
         <v>146</v>
       </c>

</xml_diff>